<commit_message>
Battery price filled in: OVONIC 2S 1100 mAh pair, $26.99
</commit_message>
<xml_diff>
--- a/docs/vendor-orders/all-vendors.xlsx
+++ b/docs/vendor-orders/all-vendors.xlsx
@@ -4018,7 +4018,9 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="n">
+        <v>26.99</v>
+      </c>
       <c r="D5" s="2">
         <f>B5*C5</f>
         <v/>
@@ -4030,7 +4032,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Drone; Battery; Pack of 2. High-voltage type, XT30 plug, 60C.</t>
+          <t>Drone; Battery; Pack of 2, $13.50 a battery. High-voltage type (charge to 4.35 V a cell), XT30 plug, 60C.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
Motors: Pyrodrone teal/pink listing, the gold/orange one is sold out
</commit_message>
<xml_diff>
--- a/docs/vendor-orders/all-vendors.xlsx
+++ b/docs/vendor-orders/all-vendors.xlsx
@@ -3782,7 +3782,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RCINPower GTS V3 1303 8000KV Plus</t>
+          <t>RCINPower GTS V3 1303 8000KV Plus (teal/pink)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -3797,17 +3797,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>RCINPower GTS V3 1303 8000KV Plus</t>
+          <t>RCINPower GTS V3 1303 8000KV Plus (teal/pink)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Drone; Motor; In stock 2026-10-13. A fifth as a spare is worth considering</t>
+          <t>Drone; Motor; Teal/pink, in stock 2026-10-15. The gold/orange colour is sold out; same motor.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://pyrodrone.com/products/rcinpower-gts-v3-1303-8000kv-plus-2-3-inch-cinewhoop-micro-motor-gold-orange</t>
+          <t>https://pyrodrone.com/products/rcinpower-gts-v3-1303-8000kv-plus-2-3-inch-cinewhoop-micro-motor-teal-pink</t>
         </is>
       </c>
       <c r="H2" s="2">

</xml_diff>